<commit_message>
Add quick-reference math block to SCORING_GUIDE (docs only)
Four formula lines plus a worked example between the band table and the
rubrics; no scoring logic changed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CFoRmmyZBAk7VkisRgH6G2
</commit_message>
<xml_diff>
--- a/Part-Supplier Risk Model/Part_Supplier_Risk_Model.xlsx
+++ b/Part-Supplier Risk Model/Part_Supplier_Risk_Model.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="323">
   <si>
     <t xml:space="preserve">PART-SUPPLIER RISK MODEL</t>
   </si>
@@ -575,6 +575,24 @@
   </si>
   <si>
     <t xml:space="preserve">Cutoffs follow the standard 5x5 risk-matrix convention (ISO 31000 / IEC 31010): 15-25 red, 7-14 yellow, 1-6 green.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THE MATH (quick reference)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.  Adjusted supplier scores (SUPPLIERS sheet):  Stability_Adj = MIN(5, Stability_Base + number of yellow flags tagged 'Stability').  External_Adj works the same with 'External' flags.  No flags -&gt; adjusted = base.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.  Likelihood (1-5) = 25% x Sourcing_Backup + 25% x Quality_Compliance + 20% x Capacity + 20% x Stability_Adj + 10% x External_Adj.  Left blank until all five criteria have a value.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.  Risk_Score (1-25) = Likelihood x Impact.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.  Risk_Band:  any red flag on the supplier -&gt; CRITICAL (FLAG).  Otherwise: missing scores -&gt; NOT SCORED;  Risk &gt;= 15 -&gt; CRITICAL;  Risk &gt;= 7 -&gt; MONITOR;  below 7 -&gt; LOW.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worked example (the pork belly row):  Sourcing 5, Quality 4, Capacity 3, Stability 4, External 4  -&gt;  1.25 + 1.00 + 0.60 + 0.80 + 0.40  =  Likelihood 4.1.  Impact 5  -&gt;  Risk 20.5  -&gt;  CRITICAL.</t>
   </si>
   <si>
     <t xml:space="preserve">SOURCING &amp; BACKUP  (part-level)</t>
@@ -25643,7 +25661,7 @@
     <tabColor rgb="FF548235"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
@@ -25808,587 +25826,587 @@
         <v>177</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
+    <row r="24" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="44" t="s">
         <v>178</v>
       </c>
-      <c r="C24" s="33" t="s">
+      <c r="B24" s="44"/>
+      <c r="C24" s="44"/>
+    </row>
+    <row r="25" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="44" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" s="36" t="s">
+      <c r="B25" s="44"/>
+      <c r="C25" s="44"/>
+    </row>
+    <row r="26" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="44" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="C26" s="36" t="s">
+      <c r="B26" s="44"/>
+      <c r="C26" s="44"/>
+    </row>
+    <row r="27" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="44" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="31" t="n">
-        <v>5</v>
-      </c>
-      <c r="C27" s="36" t="s">
+      <c r="B27" s="44"/>
+      <c r="C27" s="44"/>
+    </row>
+    <row r="28" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="44" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="s">
+      <c r="B28" s="44"/>
+      <c r="C28" s="44"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="C30" s="33" t="s">
-        <v>179</v>
-      </c>
-    </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" s="36" t="s">
+      <c r="A31" s="5" t="s">
         <v>184</v>
+      </c>
+      <c r="C31" s="33" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C32" s="36" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" s="36" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="C33" s="36" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C34" s="43" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C35" s="43" t="s">
+      <c r="C34" s="36" t="s">
         <v>188</v>
       </c>
     </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="10" t="s">
+        <v>189</v>
+      </c>
+    </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="10" t="s">
-        <v>189</v>
+      <c r="A37" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C37" s="33" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="C38" s="33" t="s">
-        <v>179</v>
+      <c r="A38" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" s="36" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C39" s="36" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="31" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C40" s="36" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="31" t="n">
-        <v>5</v>
-      </c>
-      <c r="C41" s="36" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="10" t="s">
+      <c r="C41" s="43" t="s">
         <v>193</v>
       </c>
     </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C42" s="43" t="s">
+        <v>194</v>
+      </c>
+    </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="C44" s="33" t="s">
-        <v>179</v>
+      <c r="A44" s="10" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C45" s="36" t="s">
-        <v>194</v>
+      <c r="A45" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C45" s="33" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C46" s="36" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C47" s="36" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="C47" s="36" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C48" s="43" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C49" s="43" t="s">
+      <c r="C48" s="36" t="s">
         <v>198</v>
       </c>
     </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="10" t="s">
+        <v>199</v>
+      </c>
+    </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="10" t="s">
-        <v>199</v>
+      <c r="A51" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C51" s="33" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="C52" s="33" t="s">
-        <v>179</v>
+      <c r="A52" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="36" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C53" s="36" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="31" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C54" s="36" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="31" t="n">
-        <v>5</v>
-      </c>
-      <c r="C55" s="36" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="10" t="s">
+      <c r="C55" s="43" t="s">
         <v>203</v>
       </c>
     </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C56" s="43" t="s">
+        <v>204</v>
+      </c>
+    </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="C58" s="33" t="s">
-        <v>179</v>
+      <c r="A58" s="10" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C59" s="36" t="s">
-        <v>204</v>
+      <c r="A59" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C59" s="33" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C60" s="36" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C61" s="36" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="C61" s="36" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="10" t="s">
-        <v>207</v>
+      <c r="C62" s="36" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="33" t="s">
-        <v>208</v>
-      </c>
-      <c r="C64" s="33" t="s">
+      <c r="A64" s="10" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="36" t="s">
+      <c r="A65" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C65" s="33" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="36" t="s">
         <v>210</v>
       </c>
-      <c r="C65" s="36" t="s">
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C67" s="36" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="36" t="s">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="C68" s="36" t="s">
         <v>212</v>
       </c>
-      <c r="C66" s="36" t="s">
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="10" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="36" t="s">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="33" t="s">
         <v>214</v>
       </c>
-      <c r="C67" s="36" t="s">
+      <c r="C71" s="33" t="s">
         <v>215</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="36" t="s">
-        <v>216</v>
-      </c>
-      <c r="C68" s="36" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="36" t="s">
-        <v>218</v>
-      </c>
-      <c r="C69" s="36" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="36" t="s">
-        <v>220</v>
-      </c>
-      <c r="C70" s="36" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="36" t="s">
-        <v>222</v>
-      </c>
-      <c r="C71" s="36" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="36" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C72" s="36" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="36" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="C73" s="36" t="s">
-        <v>227</v>
+        <v>219</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="36" t="s">
+        <v>220</v>
+      </c>
+      <c r="C74" s="36" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="10" t="s">
-        <v>228</v>
+      <c r="A75" s="36" t="s">
+        <v>222</v>
+      </c>
+      <c r="C75" s="36" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="33" t="s">
-        <v>229</v>
-      </c>
-      <c r="C76" s="33" t="s">
-        <v>230</v>
+      <c r="A76" s="36" t="s">
+        <v>224</v>
+      </c>
+      <c r="C76" s="36" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="36" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="C77" s="36" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="36" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="C78" s="36" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="36" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="C79" s="36" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="36" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="C80" s="36" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="36" t="s">
-        <v>239</v>
-      </c>
-      <c r="C81" s="36" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="36" t="s">
-        <v>241</v>
-      </c>
-      <c r="C82" s="36" t="s">
-        <v>242</v>
+      <c r="A82" s="10" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="36" t="s">
-        <v>243</v>
-      </c>
-      <c r="C83" s="36" t="s">
-        <v>244</v>
+      <c r="A83" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="C83" s="33" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="36" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="C84" s="36" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="36" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="C85" s="36" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="36" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="C86" s="36" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="36" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="C87" s="36" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="36" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="C88" s="36" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="36" t="s">
+        <v>247</v>
+      </c>
+      <c r="C89" s="36" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="36" t="s">
+        <v>249</v>
+      </c>
+      <c r="C90" s="36" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="36" t="s">
+        <v>251</v>
+      </c>
+      <c r="C91" s="36" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="36" t="s">
+        <v>253</v>
+      </c>
+      <c r="C92" s="36" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="36" t="s">
         <v>255</v>
       </c>
-      <c r="C89" s="36" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="10" t="s">
+      <c r="C93" s="36" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="44" t="s">
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="B92" s="44"/>
-      <c r="C92" s="44"/>
-    </row>
-    <row r="93" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="44" t="s">
+      <c r="C94" s="36" t="s">
         <v>258</v>
       </c>
-      <c r="B93" s="44"/>
-      <c r="C93" s="44"/>
-    </row>
-    <row r="94" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A94" s="44" t="s">
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="36" t="s">
         <v>259</v>
       </c>
-      <c r="B94" s="44"/>
-      <c r="C94" s="44"/>
-    </row>
-    <row r="95" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A95" s="44" t="s">
+      <c r="C95" s="36" t="s">
         <v>260</v>
       </c>
-      <c r="B95" s="44"/>
-      <c r="C95" s="44"/>
-    </row>
-    <row r="96" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A96" s="44" t="s">
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="36" t="s">
         <v>261</v>
       </c>
-      <c r="B96" s="44"/>
-      <c r="C96" s="44"/>
-    </row>
-    <row r="97" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A97" s="44" t="s">
+      <c r="C96" s="36" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="B97" s="44"/>
-      <c r="C97" s="44"/>
-    </row>
-    <row r="98" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A98" s="44" t="s">
+    </row>
+    <row r="99" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A99" s="44" t="s">
         <v>263</v>
       </c>
-      <c r="B98" s="44"/>
-      <c r="C98" s="44"/>
-    </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="10" t="s">
+      <c r="B99" s="44"/>
+      <c r="C99" s="44"/>
+    </row>
+    <row r="100" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A100" s="44" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="101" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B100" s="44"/>
+      <c r="C100" s="44"/>
+    </row>
+    <row r="101" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="44" t="s">
         <v>265</v>
       </c>
       <c r="B101" s="44"/>
       <c r="C101" s="44"/>
     </row>
-    <row r="102" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="44" t="s">
         <v>266</v>
       </c>
       <c r="B102" s="44"/>
       <c r="C102" s="44"/>
     </row>
-    <row r="103" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="44" t="s">
         <v>267</v>
       </c>
       <c r="B103" s="44"/>
       <c r="C103" s="44"/>
     </row>
-    <row r="104" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="44" t="s">
         <v>268</v>
       </c>
       <c r="B104" s="44"/>
       <c r="C104" s="44"/>
     </row>
-    <row r="105" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="44" t="s">
         <v>269</v>
       </c>
       <c r="B105" s="44"/>
       <c r="C105" s="44"/>
     </row>
-    <row r="106" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A106" s="44" t="s">
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="B106" s="44"/>
-      <c r="C106" s="44"/>
-    </row>
-    <row r="107" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A107" s="44" t="s">
+    </row>
+    <row r="108" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A108" s="44" t="s">
         <v>271</v>
       </c>
-      <c r="B107" s="44"/>
-      <c r="C107" s="44"/>
-    </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="10" t="s">
+      <c r="B108" s="44"/>
+      <c r="C108" s="44"/>
+    </row>
+    <row r="109" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A109" s="44" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="110" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B109" s="44"/>
+      <c r="C109" s="44"/>
+    </row>
+    <row r="110" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="44" t="s">
         <v>273</v>
       </c>
       <c r="B110" s="44"/>
       <c r="C110" s="44"/>
     </row>
-    <row r="111" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="44" t="s">
         <v>274</v>
       </c>
       <c r="B111" s="44"/>
       <c r="C111" s="44"/>
     </row>
-    <row r="112" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="44" t="s">
         <v>275</v>
       </c>
       <c r="B112" s="44"/>
       <c r="C112" s="44"/>
     </row>
-    <row r="113" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="44" t="s">
         <v>276</v>
       </c>
       <c r="B113" s="44"/>
       <c r="C113" s="44"/>
     </row>
-    <row r="114" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="44" t="s">
         <v>277</v>
       </c>
@@ -26435,43 +26453,83 @@
       <c r="B121" s="44"/>
       <c r="C121" s="44"/>
     </row>
-    <row r="122" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A122" s="44" t="s">
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="B122" s="44"/>
-      <c r="C122" s="44"/>
-    </row>
-    <row r="123" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A123" s="44" t="s">
-        <v>285</v>
-      </c>
-      <c r="B123" s="44"/>
-      <c r="C123" s="44"/>
     </row>
     <row r="124" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="44" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B124" s="44"/>
       <c r="C124" s="44"/>
     </row>
+    <row r="125" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A125" s="44" t="s">
+        <v>286</v>
+      </c>
+      <c r="B125" s="44"/>
+      <c r="C125" s="44"/>
+    </row>
+    <row r="126" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A126" s="44" t="s">
+        <v>287</v>
+      </c>
+      <c r="B126" s="44"/>
+      <c r="C126" s="44"/>
+    </row>
+    <row r="127" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A127" s="44" t="s">
+        <v>288</v>
+      </c>
+      <c r="B127" s="44"/>
+      <c r="C127" s="44"/>
+    </row>
+    <row r="128" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A128" s="44" t="s">
+        <v>289</v>
+      </c>
+      <c r="B128" s="44"/>
+      <c r="C128" s="44"/>
+    </row>
+    <row r="129" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A129" s="44" t="s">
+        <v>290</v>
+      </c>
+      <c r="B129" s="44"/>
+      <c r="C129" s="44"/>
+    </row>
+    <row r="130" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A130" s="44" t="s">
+        <v>291</v>
+      </c>
+      <c r="B130" s="44"/>
+      <c r="C130" s="44"/>
+    </row>
+    <row r="131" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A131" s="44" t="s">
+        <v>292</v>
+      </c>
+      <c r="B131" s="44"/>
+      <c r="C131" s="44"/>
+    </row>
   </sheetData>
-  <mergeCells count="27">
-    <mergeCell ref="A92:C92"/>
-    <mergeCell ref="A93:C93"/>
-    <mergeCell ref="A94:C94"/>
-    <mergeCell ref="A95:C95"/>
-    <mergeCell ref="A96:C96"/>
-    <mergeCell ref="A97:C97"/>
-    <mergeCell ref="A98:C98"/>
+  <mergeCells count="32">
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A99:C99"/>
+    <mergeCell ref="A100:C100"/>
     <mergeCell ref="A101:C101"/>
     <mergeCell ref="A102:C102"/>
     <mergeCell ref="A103:C103"/>
     <mergeCell ref="A104:C104"/>
     <mergeCell ref="A105:C105"/>
-    <mergeCell ref="A106:C106"/>
-    <mergeCell ref="A107:C107"/>
+    <mergeCell ref="A108:C108"/>
+    <mergeCell ref="A109:C109"/>
     <mergeCell ref="A110:C110"/>
     <mergeCell ref="A111:C111"/>
     <mergeCell ref="A112:C112"/>
@@ -26482,9 +26540,14 @@
     <mergeCell ref="A119:C119"/>
     <mergeCell ref="A120:C120"/>
     <mergeCell ref="A121:C121"/>
-    <mergeCell ref="A122:C122"/>
-    <mergeCell ref="A123:C123"/>
     <mergeCell ref="A124:C124"/>
+    <mergeCell ref="A125:C125"/>
+    <mergeCell ref="A126:C126"/>
+    <mergeCell ref="A127:C127"/>
+    <mergeCell ref="A128:C128"/>
+    <mergeCell ref="A129:C129"/>
+    <mergeCell ref="A130:C130"/>
+    <mergeCell ref="A131:C131"/>
   </mergeCells>
   <conditionalFormatting sqref="B14">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -26520,25 +26583,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26549,16 +26612,16 @@
         <v>1</v>
       </c>
       <c r="C2" s="45" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="D2" s="45" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="E2" s="45" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="G2" s="45" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="H2" s="45" t="s">
         <v>155</v>
@@ -26566,19 +26629,19 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="45" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="B3" s="45" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D3" s="45" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="E3" s="45" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="G3" s="45" t="s">
         <v>124</v>
@@ -26595,16 +26658,16 @@
         <v>3</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="D4" s="45" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="E4" s="45" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="G4" s="45" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="H4" s="45" t="s">
         <v>67</v>
@@ -26618,16 +26681,16 @@
         <v>4</v>
       </c>
       <c r="C5" s="45" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="D5" s="45" t="s">
+        <v>307</v>
+      </c>
+      <c r="E5" s="45" t="s">
         <v>301</v>
       </c>
-      <c r="E5" s="45" t="s">
-        <v>295</v>
-      </c>
       <c r="G5" s="45" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="H5" s="45" t="s">
         <v>160</v>
@@ -26638,16 +26701,16 @@
         <v>5</v>
       </c>
       <c r="C6" s="45" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="D6" s="45" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="E6" s="45" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="G6" s="45" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="H6" s="45" t="s">
         <v>162</v>
@@ -26655,94 +26718,94 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C7" s="45" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="D7" s="45" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="E7" s="45" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="G7" s="45" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C8" s="45" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="D8" s="45" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="E8" s="45" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="45" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="D9" s="45" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="E9" s="45" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C10" s="45" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="D10" s="45" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="E10" s="45" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D11" s="45" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="E11" s="45" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D12" s="45" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E12" s="45" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D13" s="45" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="E13" s="45" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D14" s="45" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="E14" s="45" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D15" s="45" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="E15" s="45" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="46" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="B18" s="46"/>
       <c r="C18" s="46"/>

</xml_diff>